<commit_message>
xgboost as base method in progress
</commit_message>
<xml_diff>
--- a/data/LLMSurveys_Configurations.xlsx
+++ b/data/LLMSurveys_Configurations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Current\Work\LLMExpectations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2362E3-0BE8-4CD9-B4BB-66D900C4B4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910AA88B-B280-4527-A945-1EE1855025F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2800" yWindow="2800" windowWidth="14400" windowHeight="7270" xr2:uid="{1E49B1B9-B097-4895-90AA-09F755188166}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1E49B1B9-B097-4895-90AA-09F755188166}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="37">
   <si>
     <t>UsdRub</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>QWEN 3.8 (reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>QWEN 3.8 (+news +rlms e, 7d)</t>
   </si>
 </sst>
 </file>
@@ -182,7 +185,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -205,11 +208,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -219,11 +237,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -554,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF250728-16E4-438D-A8DD-F8C642EF43D3}">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.81640625" customWidth="1"/>
@@ -1434,8 +1473,51 @@
         <v>10</v>
       </c>
     </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B1:K25">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Да"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>"Нет"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26:K26">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Да"</formula>
     </cfRule>

</xml_diff>

<commit_message>
llm surveys configuration fixed
</commit_message>
<xml_diff>
--- a/data/LLMSurveys_Configurations.xlsx
+++ b/data/LLMSurveys_Configurations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Current\Work\LLMExpectations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9321CFF-C47A-46FC-B78F-43A01F44D26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35ECDC4-14A5-4EFC-831C-BD98C005D776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1E49B1B9-B097-4895-90AA-09F755188166}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="42">
   <si>
     <t>UsdRub</t>
   </si>
@@ -151,6 +151,15 @@
   </si>
   <si>
     <t>Gemma 3 27b (news only, 7d)</t>
+  </si>
+  <si>
+    <t>Gemma 3 27b (+news +rlms e, 7d)</t>
+  </si>
+  <si>
+    <t>LLama 70b (news only, 7d)</t>
+  </si>
+  <si>
+    <t>LLama 70b (+news +rlms e, 7d)</t>
   </si>
 </sst>
 </file>
@@ -248,7 +257,47 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -599,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF250728-16E4-438D-A8DD-F8C642EF43D3}">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.81640625" customWidth="1"/>
@@ -1584,8 +1633,129 @@
         <v>10</v>
       </c>
     </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:K27">
+  <conditionalFormatting sqref="B1:K28">
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+      <formula>"Да"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+      <formula>"Нет"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29:K29">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+      <formula>"Да"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+      <formula>"Нет"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30:K30">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Да"</formula>
     </cfRule>
@@ -1593,7 +1763,7 @@
       <formula>"Нет"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28:K28">
+  <conditionalFormatting sqref="B31:K31">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Да"</formula>
     </cfRule>

</xml_diff>

<commit_message>
added logic for multiple averaging of models
</commit_message>
<xml_diff>
--- a/data/LLMSurveys_Configurations.xlsx
+++ b/data/LLMSurveys_Configurations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Current\Work\LLMExpectations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D416A6AB-F389-4420-9B5B-845FA3A10C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7774FE-3E4B-490D-82B1-654041699554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1E49B1B9-B097-4895-90AA-09F755188166}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="82">
   <si>
     <t>UsdRub</t>
   </si>
@@ -175,6 +175,111 @@
   </si>
   <si>
     <t>LLama 70b (news + hard data, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (все данные + IE - markers, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.6 (без RLMS, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (без RLMS + IE - markers, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (RLMS pass - markers - IE - , -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (без RLMS без IE без маркеров + общ инфо, -7d от Инфом</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (без RLMS без IE + ключ, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (RLMS pass -IE + ключ, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news + RLMS pass -IE + ключ, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news - RLMS - IE + ключ, 7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news + RLMS e - IE + ключ, 7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news + RLMS e - IE - ключ, 7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (RLMS e -news -IE -ключ, 7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (-RLMS +news -IE -ключ, 7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS e +news -markers, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS e +news +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS full  +news +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.6 (только RLMS, -7d от Инфом)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS full  -news +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS e  -news +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS full  +anews +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+RLMS e  +anews +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news only, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+news +reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (reg inf, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (+news +rlms e, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (rlms e, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_Gemma 3 27b (news only, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_Gemma 3 27b (+news +rlms e, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_LLama 70b (news only, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_LLama 70b (+news +rlms e, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_Gemma 3 27b (hard data, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_LLama 70b (hard data, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_QWEN 3.8 (news + hard data, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_Gemma 3 27b (news + hard data, 7d)</t>
+  </si>
+  <si>
+    <t>Avg_LLama 70b (news + hard data, 7d)</t>
   </si>
 </sst>
 </file>
@@ -306,47 +411,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -697,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF250728-16E4-438D-A8DD-F8C642EF43D3}">
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.81640625" customWidth="1"/>
@@ -1962,24 +2027,1233 @@
         <v>10</v>
       </c>
     </row>
+    <row r="37" spans="1:11">
+      <c r="A37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
+      <c r="A40" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="A44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45" t="s">
+        <v>55</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="A46" t="s">
+        <v>56</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="A47" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="A48" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11">
+      <c r="A49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11">
+      <c r="A50" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11">
+      <c r="A51" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11">
+      <c r="A52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11">
+      <c r="A53" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11">
+      <c r="A54" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11">
+      <c r="A55" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11">
+      <c r="A56" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11">
+      <c r="A57" t="s">
+        <v>67</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11">
+      <c r="A58" t="s">
+        <v>68</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11">
+      <c r="A59" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11">
+      <c r="A60" t="s">
+        <v>70</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11">
+      <c r="A61" t="s">
+        <v>71</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11">
+      <c r="A62" t="s">
+        <v>72</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11">
+      <c r="A63" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11">
+      <c r="A64" t="s">
+        <v>74</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11">
+      <c r="A65" t="s">
+        <v>75</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11">
+      <c r="A66" t="s">
+        <v>76</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11">
+      <c r="A67" t="s">
+        <v>77</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E67" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I67" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J67" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K67" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11">
+      <c r="A68" t="s">
+        <v>78</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E68" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I68" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J68" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K68" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11">
+      <c r="A69" t="s">
+        <v>79</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H69" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I69" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J69" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K69" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11">
+      <c r="A70" t="s">
+        <v>80</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I70" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J70" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K70" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11">
+      <c r="A71" t="s">
+        <v>81</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I71" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J71" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K71" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:K33">
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
-      <formula>"Да"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
-      <formula>"Нет"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34:K34">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
-      <formula>"Да"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
-      <formula>"Нет"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B35:K35">
+  <conditionalFormatting sqref="B1:K36">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Да"</formula>
     </cfRule>
@@ -1987,7 +3261,7 @@
       <formula>"Нет"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B36:K36">
+  <conditionalFormatting sqref="B37:K71">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Да"</formula>
     </cfRule>

</xml_diff>